<commit_message>
gerbers, pcb, and sch all correct now. Improved docs
</commit_message>
<xml_diff>
--- a/bom/BT_Switch_Mechanical_BOM.xlsx
+++ b/bom/BT_Switch_Mechanical_BOM.xlsx
@@ -890,7 +890,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C4, C12</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -914,11 +914,11 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Charger VBUS input decoupling.</t>
+          <t>C4: charger VBUS input decoupling. C12: EN-to-GND, forms an RC reset delay with R5 (10 k x 1 uF).</t>
         </is>
       </c>
     </row>

</xml_diff>